<commit_message>
extracted raw data, 5-year average, and gini-interpolated data for all countries at once.
</commit_message>
<xml_diff>
--- a/XLSX_DATA/RAW_DATA/BGD_raw_data.xlsx
+++ b/XLSX_DATA/RAW_DATA/BGD_raw_data.xlsx
@@ -449,12 +449,12 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>gini</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>log_gdp_pc</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>gini</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -503,10 +503,10 @@
         <v>537.931946643983</v>
       </c>
       <c r="G2" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="H2" t="n">
         <v>6.287732058934044</v>
-      </c>
-      <c r="H2" t="n">
-        <v>32.9</v>
       </c>
       <c r="I2" t="n">
         <v>23.5808244521571</v>
@@ -543,10 +543,10 @@
       <c r="F3" t="n">
         <v>552.077107138767</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
         <v>6.313687723367389</v>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>21.6839165728619</v>
       </c>
@@ -582,10 +582,10 @@
       <c r="F4" t="n">
         <v>566.271140847632</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
         <v>6.339073010930571</v>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>21.8626700944451</v>
       </c>
@@ -623,10 +623,10 @@
       <c r="F5" t="n">
         <v>584.448175174047</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
         <v>6.37066811175281</v>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
         <v>22.6607423702209</v>
       </c>
@@ -664,10 +664,10 @@
       <c r="F6" t="n">
         <v>600.232323162952</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
         <v>6.397316785543117</v>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>22.3758655367007</v>
       </c>
@@ -706,10 +706,10 @@
         <v>620.560472822105</v>
       </c>
       <c r="G7" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="H7" t="n">
         <v>6.430623058110431</v>
-      </c>
-      <c r="H7" t="n">
-        <v>33.4</v>
       </c>
       <c r="I7" t="n">
         <v>22.2793826819325</v>
@@ -748,10 +748,10 @@
       <c r="F8" t="n">
         <v>641.288922876274</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
         <v>6.463480093085436</v>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
         <v>22.5838118742213</v>
       </c>
@@ -789,10 +789,10 @@
       <c r="F9" t="n">
         <v>655.672139362272</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
         <v>6.485660876451147</v>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
         <v>22.8392543728467</v>
       </c>
@@ -830,10 +830,10 @@
       <c r="F10" t="n">
         <v>676.826252046427</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
         <v>6.517414596024433</v>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>22.4741487860882</v>
       </c>
@@ -871,10 +871,10 @@
       <c r="F11" t="n">
         <v>702.656357081873</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
         <v>6.554867948800887</v>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>22.7797200060528</v>
       </c>
@@ -913,10 +913,10 @@
         <v>739.203718353409</v>
       </c>
       <c r="G12" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="H12" t="n">
         <v>6.605573550554825</v>
-      </c>
-      <c r="H12" t="n">
-        <v>33.2</v>
       </c>
       <c r="I12" t="n">
         <v>23.2998442190711</v>
@@ -955,10 +955,10 @@
       <c r="F13" t="n">
         <v>779.419570444998</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
         <v>6.658549502218567</v>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
         <v>24.0953205119221</v>
       </c>
@@ -996,10 +996,10 @@
       <c r="F14" t="n">
         <v>825.508229964537</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
         <v>6.715999232982851</v>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
         <v>24.5005410079343</v>
       </c>
@@ -1037,10 +1037,10 @@
       <c r="F15" t="n">
         <v>866.45815762135</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
         <v>6.764413819035702</v>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>24.7270013036793</v>
       </c>
@@ -1078,10 +1078,10 @@
       <c r="F16" t="n">
         <v>901.729626251937</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
         <v>6.804314725962496</v>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
         <v>25.2955721814431</v>
       </c>
@@ -1120,10 +1120,10 @@
         <v>943.6642286423599</v>
       </c>
       <c r="G17" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="H17" t="n">
         <v>6.849770412875309</v>
-      </c>
-      <c r="H17" t="n">
-        <v>32.1</v>
       </c>
       <c r="I17" t="n">
         <v>24.9564767264585</v>
@@ -1162,10 +1162,10 @@
       <c r="F18" t="n">
         <v>995.579947155662</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
         <v>6.903325428823803</v>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
         <v>25.0452996007551</v>
       </c>
@@ -1203,10 +1203,10 @@
       <c r="F19" t="n">
         <v>1050.39140404066</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
         <v>6.956918139444686</v>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
         <v>25.3099593902625</v>
       </c>
@@ -1244,10 +1244,10 @@
       <c r="F20" t="n">
         <v>1103.15695907123</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
         <v>7.005931311098014</v>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>26.3070701636507</v>
       </c>
@@ -1283,10 +1283,10 @@
       <c r="F21" t="n">
         <v>1159.40753475981</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
         <v>7.055664407728581</v>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
         <v>26.3110467833576</v>
       </c>
@@ -1324,10 +1324,10 @@
       <c r="F22" t="n">
         <v>1224.38647668165</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
         <v>7.110195162156987</v>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
         <v>26.8313948329541</v>
       </c>
@@ -1366,10 +1366,10 @@
         <v>1299.83091360792</v>
       </c>
       <c r="G23" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="H23" t="n">
         <v>7.169989468534807</v>
-      </c>
-      <c r="H23" t="n">
-        <v>32.4</v>
       </c>
       <c r="I23" t="n">
         <v>31.0691513830358</v>
@@ -1408,10 +1408,10 @@
       <c r="F24" t="n">
         <v>1373.75363740186</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
         <v>7.225302153504579</v>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>31.2482919641603</v>
       </c>
@@ -1449,10 +1449,10 @@
       <c r="F25" t="n">
         <v>1462.25050255713</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
         <v>7.287731968010632</v>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>31.9828135899766</v>
       </c>
@@ -1490,10 +1490,10 @@
       <c r="F26" t="n">
         <v>1564.20802445636</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
         <v>7.355134920224906</v>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
         <v>32.8525491977868</v>
       </c>
@@ -1531,10 +1531,10 @@
       <c r="F27" t="n">
         <v>1604.6659234742</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
         <v>7.380670866530346</v>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
         <v>32.9115650824449</v>
       </c>
@@ -1572,10 +1572,10 @@
       <c r="F28" t="n">
         <v>1702.08028414189</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
         <v>7.439606478491974</v>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
         <v>33.3160943869001</v>
       </c>
@@ -1614,10 +1614,10 @@
         <v>1804.3493461776</v>
       </c>
       <c r="G29" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="H29" t="n">
         <v>7.49795533274916</v>
-      </c>
-      <c r="H29" t="n">
-        <v>30.9</v>
       </c>
       <c r="I29" t="n">
         <v>33.9200804971876</v>
@@ -1656,10 +1656,10 @@
       <c r="F30" t="n">
         <v>1885.37733613545</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
         <v>7.541883258170298</v>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
         <v>34.5942721606063</v>
       </c>
@@ -1697,10 +1697,10 @@
       <c r="F31" t="n">
         <v>1941.27874360025</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
         <v>7.571102181101636</v>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
         <v>34.0971743458877</v>
       </c>

</xml_diff>

<commit_message>
Extracted wgi data for cc, va and ge indicators, merged to each country's primary dataset.
</commit_message>
<xml_diff>
--- a/XLSX_DATA/RAW_DATA/BGD_raw_data.xlsx
+++ b/XLSX_DATA/RAW_DATA/BGD_raw_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,21 @@
           <t>palma_ratio</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>va_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>cc_score</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ge_score</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -521,8 +536,11 @@
         <v>21.3383159101032</v>
       </c>
       <c r="M2" t="n">
-        <v>4.358999037536092</v>
-      </c>
+        <v>3.878679750223015</v>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -562,8 +580,11 @@
         <v>21.661231550566</v>
       </c>
       <c r="M3" t="n">
-        <v>4.538537549407114</v>
-      </c>
+        <v>4.140221402214022</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,7 +624,16 @@
         <v>21.9780786680138</v>
       </c>
       <c r="M4" t="n">
-        <v>4.465686274509804</v>
+        <v>4.153061224489796</v>
+      </c>
+      <c r="N4" t="n">
+        <v>51.29</v>
+      </c>
+      <c r="O4" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="P4" t="n">
+        <v>35.57</v>
       </c>
     </row>
     <row r="5">
@@ -644,8 +674,11 @@
         <v>22.2953437419401</v>
       </c>
       <c r="M5" t="n">
-        <v>4.405458089668616</v>
-      </c>
+        <v>4.171802054154995</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -687,7 +720,16 @@
         <v>22.6195132518384</v>
       </c>
       <c r="M6" t="n">
-        <v>4.326254826254826</v>
+        <v>4.175257731958763</v>
+      </c>
+      <c r="N6" t="n">
+        <v>50.75</v>
+      </c>
+      <c r="O6" t="n">
+        <v>30.18</v>
+      </c>
+      <c r="P6" t="n">
+        <v>40.75</v>
       </c>
     </row>
     <row r="7">
@@ -730,8 +772,11 @@
         <v>22.957073677202</v>
       </c>
       <c r="M7" t="n">
-        <v>4.302123552123552</v>
-      </c>
+        <v>4.226755218216319</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -773,7 +818,16 @@
         <v>23.3145114975244</v>
       </c>
       <c r="M8" t="n">
-        <v>4.251681075888569</v>
+        <v>4.245229007633588</v>
+      </c>
+      <c r="N8" t="n">
+        <v>49.11</v>
+      </c>
+      <c r="O8" t="n">
+        <v>24.78</v>
+      </c>
+      <c r="P8" t="n">
+        <v>34.4</v>
       </c>
     </row>
     <row r="9">
@@ -816,8 +870,11 @@
         <v>23.6999214768623</v>
       </c>
       <c r="M9" t="n">
-        <v>4.191793893129771</v>
-      </c>
+        <v>4.262906309751434</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -859,7 +916,16 @@
         <v>24.1132383547332</v>
       </c>
       <c r="M10" t="n">
-        <v>4.208453410182517</v>
+        <v>4.35631067961165</v>
+      </c>
+      <c r="N10" t="n">
+        <v>45.29</v>
+      </c>
+      <c r="O10" t="n">
+        <v>18.52</v>
+      </c>
+      <c r="P10" t="n">
+        <v>34.73</v>
       </c>
     </row>
     <row r="11">
@@ -902,7 +968,16 @@
         <v>24.5525557512625</v>
       </c>
       <c r="M11" t="n">
-        <v>4.264849074975658</v>
+        <v>4.486111111111111</v>
+      </c>
+      <c r="N11" t="n">
+        <v>44.32</v>
+      </c>
+      <c r="O11" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="P11" t="n">
+        <v>30.6</v>
       </c>
     </row>
     <row r="12">
@@ -945,7 +1020,16 @@
         <v>25.0094809886101</v>
       </c>
       <c r="M12" t="n">
-        <v>4.212003872216844</v>
+        <v>4.509452736318408</v>
+      </c>
+      <c r="N12" t="n">
+        <v>45.98</v>
+      </c>
+      <c r="O12" t="n">
+        <v>17.17</v>
+      </c>
+      <c r="P12" t="n">
+        <v>33.72</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +1072,16 @@
         <v>25.4769540701509</v>
       </c>
       <c r="M13" t="n">
-        <v>4.192642787996127</v>
+        <v>4.557114228456913</v>
+      </c>
+      <c r="N13" t="n">
+        <v>47.11</v>
+      </c>
+      <c r="O13" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="P13" t="n">
+        <v>33.94</v>
       </c>
     </row>
     <row r="14">
@@ -1031,7 +1124,16 @@
         <v>25.9479149992596</v>
       </c>
       <c r="M14" t="n">
-        <v>4.203307392996109</v>
+        <v>4.481628599801391</v>
+      </c>
+      <c r="N14" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="O14" t="n">
+        <v>18.91</v>
+      </c>
+      <c r="P14" t="n">
+        <v>32.99</v>
       </c>
     </row>
     <row r="15">
@@ -1074,7 +1176,16 @@
         <v>26.415303779311</v>
       </c>
       <c r="M15" t="n">
-        <v>4.242632612966601</v>
+        <v>4.447968285431119</v>
+      </c>
+      <c r="N15" t="n">
+        <v>47.96</v>
+      </c>
+      <c r="O15" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="P15" t="n">
+        <v>34.37</v>
       </c>
     </row>
     <row r="16">
@@ -1117,7 +1228,16 @@
         <v>26.87206041368</v>
       </c>
       <c r="M16" t="n">
-        <v>4.038973384030419</v>
+        <v>4.177251184834123</v>
+      </c>
+      <c r="N16" t="n">
+        <v>48.65</v>
+      </c>
+      <c r="O16" t="n">
+        <v>28.66</v>
+      </c>
+      <c r="P16" t="n">
+        <v>34.91</v>
       </c>
     </row>
     <row r="17">
@@ -1160,7 +1280,16 @@
         <v>27.3111249057412</v>
       </c>
       <c r="M17" t="n">
-        <v>3.970809792843691</v>
+        <v>4.06145251396648</v>
+      </c>
+      <c r="N17" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>29.41</v>
+      </c>
+      <c r="P17" t="n">
+        <v>35.5</v>
       </c>
     </row>
     <row r="18">
@@ -1203,7 +1332,16 @@
         <v>27.7254372588696</v>
       </c>
       <c r="M18" t="n">
-        <v>4.072115384615385</v>
+        <v>4.108286252354049</v>
+      </c>
+      <c r="N18" t="n">
+        <v>51.33</v>
+      </c>
+      <c r="O18" t="n">
+        <v>27.17</v>
+      </c>
+      <c r="P18" t="n">
+        <v>35.65</v>
       </c>
     </row>
     <row r="19">
@@ -1246,7 +1384,16 @@
         <v>28.1100162712427</v>
       </c>
       <c r="M19" t="n">
-        <v>3.982024597918638</v>
+        <v>3.997229916897507</v>
+      </c>
+      <c r="N19" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="O19" t="n">
+        <v>26.55</v>
+      </c>
+      <c r="P19" t="n">
+        <v>35.06</v>
       </c>
     </row>
     <row r="20">
@@ -1289,7 +1436,16 @@
         <v>28.4787972894576</v>
       </c>
       <c r="M20" t="n">
-        <v>3.965094339622642</v>
+        <v>3.959633027522936</v>
+      </c>
+      <c r="N20" t="n">
+        <v>46.13</v>
+      </c>
+      <c r="O20" t="n">
+        <v>25.16</v>
+      </c>
+      <c r="P20" t="n">
+        <v>35.81</v>
       </c>
     </row>
     <row r="21">
@@ -1332,7 +1488,16 @@
         <v>28.8407036106763</v>
       </c>
       <c r="M21" t="n">
-        <v>3.935272045028142</v>
+        <v>3.918032786885246</v>
+      </c>
+      <c r="N21" t="n">
+        <v>44.51</v>
+      </c>
+      <c r="O21" t="n">
+        <v>24.93</v>
+      </c>
+      <c r="P21" t="n">
+        <v>36.29</v>
       </c>
     </row>
     <row r="22">
@@ -1373,7 +1538,16 @@
         <v>29.1944442321013</v>
       </c>
       <c r="M22" t="n">
-        <v>3.882899628252788</v>
+        <v>3.848920863309353</v>
+      </c>
+      <c r="N22" t="n">
+        <v>43.05</v>
+      </c>
+      <c r="O22" t="n">
+        <v>23.88</v>
+      </c>
+      <c r="P22" t="n">
+        <v>38.02</v>
       </c>
     </row>
     <row r="23">
@@ -1416,7 +1590,16 @@
         <v>29.5395099477892</v>
       </c>
       <c r="M23" t="n">
-        <v>3.793418647166362</v>
+        <v>3.749338040600177</v>
+      </c>
+      <c r="N23" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="O23" t="n">
+        <v>26</v>
+      </c>
+      <c r="P23" t="n">
+        <v>38.61</v>
       </c>
     </row>
     <row r="24">
@@ -1459,7 +1642,16 @@
         <v>29.8753915517965</v>
       </c>
       <c r="M24" t="n">
-        <v>3.779398359161349</v>
+        <v>3.724956063268893</v>
+      </c>
+      <c r="N24" t="n">
+        <v>40.51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>26.26</v>
+      </c>
+      <c r="P24" t="n">
+        <v>40.96</v>
       </c>
     </row>
     <row r="25">
@@ -1502,7 +1694,16 @@
         <v>30.2015798381799</v>
       </c>
       <c r="M25" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N25" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="O25" t="n">
+        <v>26.35</v>
+      </c>
+      <c r="P25" t="n">
+        <v>40.2</v>
       </c>
     </row>
     <row r="26">
@@ -1545,7 +1746,16 @@
         <v>30.5175656009959</v>
       </c>
       <c r="M26" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N26" t="n">
+        <v>40.01</v>
+      </c>
+      <c r="O26" t="n">
+        <v>25.66</v>
+      </c>
+      <c r="P26" t="n">
+        <v>39.3</v>
       </c>
     </row>
     <row r="27">
@@ -1588,7 +1798,16 @@
         <v>30.8228396343012</v>
       </c>
       <c r="M27" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N27" t="n">
+        <v>39.52</v>
+      </c>
+      <c r="O27" t="n">
+        <v>25.58</v>
+      </c>
+      <c r="P27" t="n">
+        <v>39.73</v>
       </c>
     </row>
     <row r="28">
@@ -1631,7 +1850,16 @@
         <v>31.1168927321524</v>
       </c>
       <c r="M28" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N28" t="n">
+        <v>39.26</v>
+      </c>
+      <c r="O28" t="n">
+        <v>26.07</v>
+      </c>
+      <c r="P28" t="n">
+        <v>37.31</v>
       </c>
     </row>
     <row r="29">
@@ -1674,7 +1902,16 @@
         <v>31.3992156886061</v>
       </c>
       <c r="M29" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N29" t="n">
+        <v>38.35</v>
+      </c>
+      <c r="O29" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="P29" t="n">
+        <v>40.38</v>
       </c>
     </row>
     <row r="30">
@@ -1717,7 +1954,16 @@
         <v>31.673734726234</v>
       </c>
       <c r="M30" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N30" t="n">
+        <v>38.08</v>
+      </c>
+      <c r="O30" t="n">
+        <v>24</v>
+      </c>
+      <c r="P30" t="n">
+        <v>39.22</v>
       </c>
     </row>
     <row r="31">
@@ -1760,7 +2006,16 @@
         <v>32.1578465036834</v>
       </c>
       <c r="M31" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N31" t="n">
+        <v>36.98</v>
+      </c>
+      <c r="O31" t="n">
+        <v>23.59</v>
+      </c>
+      <c r="P31" t="n">
+        <v>40.5</v>
       </c>
     </row>
     <row r="32">
@@ -1803,7 +2058,16 @@
         <v>32.6783196323307</v>
       </c>
       <c r="M32" t="n">
-        <v>3.783759124087591</v>
+        <v>3.729111697449429</v>
+      </c>
+      <c r="N32" t="n">
+        <v>36.53</v>
+      </c>
+      <c r="O32" t="n">
+        <v>25.55</v>
+      </c>
+      <c r="P32" t="n">
+        <v>39.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>